<commit_message>
Add intermediate/advanced/pro tip columns as data-only schema.
Mirrors beginner tips for future use without changing UI or recommendation logic.

Co-authored-by: madbandi-star <madbandi-star@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/database/catalog/templates/MachineFit_카탈로그_업로드_양식.xlsx
+++ b/database/catalog/templates/MachineFit_카탈로그_업로드_양식.xlsx
@@ -19,7 +19,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_필드사전'!$A$1:$J$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_브랜드'!$A$1:$M$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03_머신'!$A$1:$Z$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03_머신'!$A$1:$AF$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_머신이미지'!$A$1:$I$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_추천설정_팁주의'!$A$1:$R$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'06_헬스장보유머신'!$A$1:$H$1</definedName>
@@ -711,7 +711,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>데이터만(미표시) — 머신 description, howTo, beginnerTips, recommendedExperience, 이미지 갤러리/alt, YouTube</t>
+          <t>데이터만(미표시) — 머신 description, howTo, beginner/intermediate/advanced/pro Tips, recommendedExperience, 이미지 갤러리/alt, YouTube</t>
         </is>
       </c>
     </row>
@@ -743,7 +743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J71"/>
+  <dimension ref="A1:J77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2362,17 +2362,17 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>recommendedExperience</t>
+          <t>intermediateTips.ko</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>추천경험레벨</t>
+          <t>중급자팁(한글)</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Recommended Experience</t>
+          <t>Intermediate Tips KO</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -2387,12 +2387,12 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>권장</t>
+          <t>선택</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>beginner/intermediate/advanced</t>
+          <t>줄바꿈 문장목록</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr">
@@ -2400,7 +2400,11 @@
           <t>03_머신</t>
         </is>
       </c>
-      <c r="J33" s="5" t="inlineStr"/>
+      <c r="J33" s="5" t="inlineStr">
+        <is>
+          <t>향후 사용</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -2410,37 +2414,37 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>hasSeat</t>
+          <t>intermediateTips.en</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>시트유무</t>
+          <t>중급자팁(영문)</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Has Seat</t>
+          <t>Intermediate Tips EN</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>추천매칭용</t>
-        </is>
-      </c>
-      <c r="F34" s="8" t="inlineStr">
-        <is>
-          <t>내부용</t>
-        </is>
-      </c>
-      <c r="G34" s="7" t="inlineStr">
-        <is>
-          <t>필수</t>
+          <t>상세(예정)</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>데이터만</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>선택</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>TRUE/FALSE</t>
+          <t>줄바꿈 문장목록</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
@@ -2448,11 +2452,7 @@
           <t>03_머신</t>
         </is>
       </c>
-      <c r="J34" s="5" t="inlineStr">
-        <is>
-          <t>화면 직접표시 없음</t>
-        </is>
-      </c>
+      <c r="J34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -2462,37 +2462,37 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>hasBackPad</t>
+          <t>advancedTips.ko</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>백패드유무</t>
+          <t>상급자팁(한글)</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Has Back Pad</t>
+          <t>Advanced Tips KO</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>추천매칭용</t>
-        </is>
-      </c>
-      <c r="F35" s="8" t="inlineStr">
-        <is>
-          <t>내부용</t>
-        </is>
-      </c>
-      <c r="G35" s="7" t="inlineStr">
-        <is>
-          <t>필수</t>
+          <t>상세(예정)</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>데이터만</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>선택</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr">
         <is>
-          <t>TRUE/FALSE</t>
+          <t>줄바꿈 문장목록</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr">
@@ -2500,7 +2500,11 @@
           <t>03_머신</t>
         </is>
       </c>
-      <c r="J35" s="5" t="inlineStr"/>
+      <c r="J35" s="5" t="inlineStr">
+        <is>
+          <t>향후 사용</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -2510,37 +2514,37 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>hasFootPlate</t>
+          <t>advancedTips.en</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>발판유무</t>
+          <t>상급자팁(영문)</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Has Foot Plate</t>
+          <t>Advanced Tips EN</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>추천매칭용</t>
-        </is>
-      </c>
-      <c r="F36" s="8" t="inlineStr">
-        <is>
-          <t>내부용</t>
-        </is>
-      </c>
-      <c r="G36" s="7" t="inlineStr">
-        <is>
-          <t>필수</t>
+          <t>상세(예정)</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>데이터만</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>선택</t>
         </is>
       </c>
       <c r="H36" s="5" t="inlineStr">
         <is>
-          <t>TRUE/FALSE</t>
+          <t>줄바꿈 문장목록</t>
         </is>
       </c>
       <c r="I36" s="5" t="inlineStr">
@@ -2558,37 +2562,37 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>hasHandle</t>
+          <t>proTips.ko</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>핸들유무</t>
+          <t>프로팁(한글)</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Has Handle</t>
+          <t>Pro Tips KO</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>추천매칭용</t>
-        </is>
-      </c>
-      <c r="F37" s="8" t="inlineStr">
-        <is>
-          <t>내부용</t>
-        </is>
-      </c>
-      <c r="G37" s="7" t="inlineStr">
-        <is>
-          <t>필수</t>
+          <t>상세(예정)</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="inlineStr">
+        <is>
+          <t>데이터만</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>선택</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
-          <t>TRUE/FALSE</t>
+          <t>줄바꿈 문장목록</t>
         </is>
       </c>
       <c r="I37" s="5" t="inlineStr">
@@ -2596,7 +2600,11 @@
           <t>03_머신</t>
         </is>
       </c>
-      <c r="J37" s="5" t="inlineStr"/>
+      <c r="J37" s="5" t="inlineStr">
+        <is>
+          <t>향후 사용</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
@@ -2606,27 +2614,27 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>romType</t>
+          <t>proTips.en</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>가동범위타입</t>
+          <t>프로팁(영문)</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>ROM Type</t>
+          <t>Pro Tips EN</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>추천기본값</t>
-        </is>
-      </c>
-      <c r="F38" s="8" t="inlineStr">
-        <is>
-          <t>내부용</t>
+          <t>상세(예정)</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="inlineStr">
+        <is>
+          <t>데이터만</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
@@ -2636,7 +2644,7 @@
       </c>
       <c r="H38" s="5" t="inlineStr">
         <is>
-          <t>fixed/variable/최대</t>
+          <t>줄바꿈 문장목록</t>
         </is>
       </c>
       <c r="I38" s="5" t="inlineStr">
@@ -2654,37 +2662,37 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>isActive</t>
+          <t>recommendedExperience</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>활성여부</t>
+          <t>추천경험레벨</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Recommended Experience</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>관리자</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="inlineStr">
-        <is>
-          <t>표시중</t>
-        </is>
-      </c>
-      <c r="G39" s="7" t="inlineStr">
-        <is>
-          <t>필수</t>
+          <t>상세(예정)</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="inlineStr">
+        <is>
+          <t>데이터만</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>권장</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
-          <t>TRUE/FALSE</t>
+          <t>beginner/intermediate/advanced</t>
         </is>
       </c>
       <c r="I39" s="5" t="inlineStr">
@@ -2697,203 +2705,195 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>이미지</t>
+          <t>머신</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>primaryImageFile / primaryImageUrl</t>
+          <t>hasSeat</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>대표이미지</t>
+          <t>시트유무</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Primary Image</t>
+          <t>Has Seat</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>검색목록/상세히어로/관리자</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="inlineStr">
-        <is>
-          <t>표시중</t>
-        </is>
-      </c>
-      <c r="G40" s="5" t="inlineStr">
-        <is>
-          <t>권장</t>
+          <t>추천매칭용</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>내부용</t>
+        </is>
+      </c>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>필수</t>
         </is>
       </c>
       <c r="H40" s="5" t="inlineStr">
         <is>
-          <t>파일명 또는 URL</t>
+          <t>TRUE/FALSE</t>
         </is>
       </c>
       <c r="I40" s="5" t="inlineStr">
         <is>
-          <t>04_머신이미지</t>
+          <t>03_머신</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>isPrimary=TRUE</t>
+          <t>화면 직접표시 없음</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>이미지</t>
+          <t>머신</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>thumbnailFile</t>
+          <t>hasBackPad</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>썸네일이미지</t>
+          <t>백패드유무</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Thumbnail</t>
+          <t>Has Back Pad</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>목록(예정)</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="inlineStr">
-        <is>
-          <t>데이터만</t>
-        </is>
-      </c>
-      <c r="G41" s="5" t="inlineStr">
-        <is>
-          <t>선택</t>
+          <t>추천매칭용</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>내부용</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>필수</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr">
         <is>
-          <t>파일명</t>
+          <t>TRUE/FALSE</t>
         </is>
       </c>
       <c r="I41" s="5" t="inlineStr">
         <is>
-          <t>04_머신이미지</t>
-        </is>
-      </c>
-      <c r="J41" s="5" t="inlineStr">
-        <is>
-          <t>없으면 대표이미지 사용</t>
-        </is>
-      </c>
+          <t>03_머신</t>
+        </is>
+      </c>
+      <c r="J41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>이미지</t>
+          <t>머신</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>galleryImageFile</t>
+          <t>hasFootPlate</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>추가이미지</t>
+          <t>발판유무</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Gallery Image</t>
+          <t>Has Foot Plate</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>갤러리(예정)</t>
-        </is>
-      </c>
-      <c r="F42" s="9" t="inlineStr">
-        <is>
-          <t>데이터만</t>
-        </is>
-      </c>
-      <c r="G42" s="5" t="inlineStr">
-        <is>
-          <t>선택</t>
+          <t>추천매칭용</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>내부용</t>
+        </is>
+      </c>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>필수</t>
         </is>
       </c>
       <c r="H42" s="5" t="inlineStr">
         <is>
-          <t>파일명/URL</t>
+          <t>TRUE/FALSE</t>
         </is>
       </c>
       <c r="I42" s="5" t="inlineStr">
         <is>
-          <t>04_머신이미지</t>
-        </is>
-      </c>
-      <c r="J42" s="5" t="inlineStr">
-        <is>
-          <t>여러 행 가능</t>
-        </is>
-      </c>
+          <t>03_머신</t>
+        </is>
+      </c>
+      <c r="J42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>이미지</t>
+          <t>머신</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>altText.ko/en</t>
+          <t>hasHandle</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>이미지대체텍스트</t>
+          <t>핸들유무</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Alt Text</t>
+          <t>Has Handle</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>접근성</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="inlineStr">
-        <is>
-          <t>데이터만</t>
-        </is>
-      </c>
-      <c r="G43" s="5" t="inlineStr">
-        <is>
-          <t>선택</t>
+          <t>추천매칭용</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>내부용</t>
+        </is>
+      </c>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>필수</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr">
         <is>
-          <t>문자열</t>
+          <t>TRUE/FALSE</t>
         </is>
       </c>
       <c r="I43" s="5" t="inlineStr">
         <is>
-          <t>04_머신이미지</t>
+          <t>03_머신</t>
         </is>
       </c>
       <c r="J43" s="5" t="inlineStr"/>
@@ -2901,32 +2901,32 @@
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>이미지</t>
+          <t>머신</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>sortOrder</t>
+          <t>romType</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>정렬순서</t>
+          <t>가동범위타입</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Sort Order</t>
+          <t>ROM Type</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>갤러리</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="inlineStr">
-        <is>
-          <t>데이터만</t>
+          <t>추천기본값</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>내부용</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
@@ -2936,44 +2936,40 @@
       </c>
       <c r="H44" s="5" t="inlineStr">
         <is>
-          <t>정수</t>
+          <t>fixed/variable/최대</t>
         </is>
       </c>
       <c r="I44" s="5" t="inlineStr">
         <is>
-          <t>04_머신이미지</t>
-        </is>
-      </c>
-      <c r="J44" s="5" t="inlineStr">
-        <is>
-          <t>0부터</t>
-        </is>
-      </c>
+          <t>03_머신</t>
+        </is>
+      </c>
+      <c r="J44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>이미지</t>
+          <t>머신</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>isPrimary</t>
+          <t>isActive</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>대표여부</t>
+          <t>활성여부</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Is Primary</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>목록/상세</t>
+          <t>관리자</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
@@ -2993,39 +2989,35 @@
       </c>
       <c r="I45" s="5" t="inlineStr">
         <is>
-          <t>04_머신이미지</t>
-        </is>
-      </c>
-      <c r="J45" s="5" t="inlineStr">
-        <is>
-          <t>머신당 TRUE 1개</t>
-        </is>
-      </c>
+          <t>03_머신</t>
+        </is>
+      </c>
+      <c r="J45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>추천설정</t>
+          <t>이미지</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>seatPosition</t>
+          <t>primaryImageFile / primaryImageUrl</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>시트 위치</t>
+          <t>대표이미지</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Seat Position</t>
+          <t>Primary Image</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>추천결과/기록/비교</t>
+          <t>검색목록/상세히어로/관리자</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
@@ -3035,165 +3027,173 @@
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>조건부</t>
+          <t>권장</t>
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr">
         <is>
-          <t>정수</t>
+          <t>파일명 또는 URL</t>
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr">
         <is>
-          <t>05_추천설정_팁주의</t>
+          <t>04_머신이미지</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
-          <t>hasSeat=TRUE일 때</t>
+          <t>isPrimary=TRUE</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>추천설정</t>
+          <t>이미지</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>backPadPosition</t>
+          <t>thumbnailFile</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>백 패드</t>
+          <t>썸네일이미지</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Back Pad</t>
+          <t>Thumbnail</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>추천결과/기록/비교</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="inlineStr">
-        <is>
-          <t>표시중</t>
+          <t>목록(예정)</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="inlineStr">
+        <is>
+          <t>데이터만</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>조건부</t>
+          <t>선택</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr">
         <is>
-          <t>정수</t>
+          <t>파일명</t>
         </is>
       </c>
       <c r="I47" s="5" t="inlineStr">
         <is>
-          <t>05_추천설정_팁주의</t>
-        </is>
-      </c>
-      <c r="J47" s="5" t="inlineStr"/>
+          <t>04_머신이미지</t>
+        </is>
+      </c>
+      <c r="J47" s="5" t="inlineStr">
+        <is>
+          <t>없으면 대표이미지 사용</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>추천설정</t>
+          <t>이미지</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>footPosition</t>
+          <t>galleryImageFile</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>발 위치</t>
+          <t>추가이미지</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Foot Position</t>
+          <t>Gallery Image</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>추천결과/기록</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="inlineStr">
-        <is>
-          <t>표시중</t>
+          <t>갤러리(예정)</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="inlineStr">
+        <is>
+          <t>데이터만</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>조건부</t>
+          <t>선택</t>
         </is>
       </c>
       <c r="H48" s="5" t="inlineStr">
         <is>
-          <t>정수</t>
+          <t>파일명/URL</t>
         </is>
       </c>
       <c r="I48" s="5" t="inlineStr">
         <is>
-          <t>05_추천설정_팁주의</t>
-        </is>
-      </c>
-      <c r="J48" s="5" t="inlineStr"/>
+          <t>04_머신이미지</t>
+        </is>
+      </c>
+      <c r="J48" s="5" t="inlineStr">
+        <is>
+          <t>여러 행 가능</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>추천설정</t>
+          <t>이미지</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>handlePosition</t>
+          <t>altText.ko/en</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>핸들 위치</t>
+          <t>이미지대체텍스트</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Handle Position</t>
+          <t>Alt Text</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>추천결과/기록/비교</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="inlineStr">
-        <is>
-          <t>표시중</t>
+          <t>접근성</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="inlineStr">
+        <is>
+          <t>데이터만</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>조건부</t>
+          <t>선택</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr">
         <is>
-          <t>정수</t>
+          <t>문자열</t>
         </is>
       </c>
       <c r="I49" s="5" t="inlineStr">
         <is>
-          <t>05_추천설정_팁주의</t>
+          <t>04_머신이미지</t>
         </is>
       </c>
       <c r="J49" s="5" t="inlineStr"/>
@@ -3201,79 +3201,79 @@
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>추천설정</t>
+          <t>이미지</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>romSetting</t>
+          <t>sortOrder</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>가동 범위</t>
+          <t>정렬순서</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>Range of Motion</t>
+          <t>Sort Order</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>추천결과/기록/비교</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="inlineStr">
-        <is>
-          <t>표시중</t>
+          <t>갤러리</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="inlineStr">
+        <is>
+          <t>데이터만</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>조건부</t>
+          <t>선택</t>
         </is>
       </c>
       <c r="H50" s="5" t="inlineStr">
         <is>
-          <t>문자열</t>
+          <t>정수</t>
         </is>
       </c>
       <c r="I50" s="5" t="inlineStr">
         <is>
-          <t>05_추천설정_팁주의</t>
+          <t>04_머신이미지</t>
         </is>
       </c>
       <c r="J50" s="5" t="inlineStr">
         <is>
-          <t>최대/부분/반/짧게/가변</t>
+          <t>0부터</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>추천설정</t>
+          <t>이미지</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>recommendedWeightKg</t>
+          <t>isPrimary</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>추천 중량</t>
+          <t>대표여부</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>Recommended Weight</t>
+          <t>Is Primary</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>추천결과/기록/비교</t>
+          <t>목록/상세</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr">
@@ -3281,22 +3281,26 @@
           <t>표시중</t>
         </is>
       </c>
-      <c r="G51" s="5" t="inlineStr">
-        <is>
-          <t>권장</t>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>필수</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">
         <is>
-          <t>숫자(kg)</t>
+          <t>TRUE/FALSE</t>
         </is>
       </c>
       <c r="I51" s="5" t="inlineStr">
         <is>
-          <t>05_추천설정_팁주의</t>
-        </is>
-      </c>
-      <c r="J51" s="5" t="inlineStr"/>
+          <t>04_머신이미지</t>
+        </is>
+      </c>
+      <c r="J51" s="5" t="inlineStr">
+        <is>
+          <t>머신당 TRUE 1개</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
@@ -3306,22 +3310,22 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>recommendedRepsMin</t>
+          <t>seatPosition</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>추천횟수최소</t>
+          <t>시트 위치</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Reps Min</t>
+          <t>Seat Position</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>추천결과</t>
+          <t>추천결과/기록/비교</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
@@ -3331,7 +3335,7 @@
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>선택</t>
+          <t>조건부</t>
         </is>
       </c>
       <c r="H52" s="5" t="inlineStr">
@@ -3346,7 +3350,7 @@
       </c>
       <c r="J52" s="5" t="inlineStr">
         <is>
-          <t>없으면 목표기반 계산</t>
+          <t>hasSeat=TRUE일 때</t>
         </is>
       </c>
     </row>
@@ -3358,22 +3362,22 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>recommendedRepsMax</t>
+          <t>backPadPosition</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>추천횟수최대</t>
+          <t>백 패드</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Reps Max</t>
+          <t>Back Pad</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>추천결과</t>
+          <t>추천결과/기록/비교</t>
         </is>
       </c>
       <c r="F53" s="6" t="inlineStr">
@@ -3383,7 +3387,7 @@
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>선택</t>
+          <t>조건부</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr">
@@ -3406,37 +3410,37 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>gender</t>
+          <t>footPosition</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>성별조건</t>
+          <t>발 위치</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Gender</t>
+          <t>Foot Position</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>추천매칭</t>
-        </is>
-      </c>
-      <c r="F54" s="8" t="inlineStr">
-        <is>
-          <t>내부용</t>
-        </is>
-      </c>
-      <c r="G54" s="7" t="inlineStr">
-        <is>
-          <t>필수</t>
+          <t>추천결과/기록</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>표시중</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>조건부</t>
         </is>
       </c>
       <c r="H54" s="5" t="inlineStr">
         <is>
-          <t>male/female</t>
+          <t>정수</t>
         </is>
       </c>
       <c r="I54" s="5" t="inlineStr">
@@ -3454,37 +3458,37 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>experienceLevel</t>
+          <t>handlePosition</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>경험레벨조건</t>
+          <t>핸들 위치</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>Experience</t>
+          <t>Handle Position</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>추천매칭</t>
-        </is>
-      </c>
-      <c r="F55" s="8" t="inlineStr">
-        <is>
-          <t>내부용</t>
-        </is>
-      </c>
-      <c r="G55" s="7" t="inlineStr">
-        <is>
-          <t>필수</t>
+          <t>추천결과/기록/비교</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="inlineStr">
+        <is>
+          <t>표시중</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>조건부</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr">
         <is>
-          <t>beginner/intermediate/advanced</t>
+          <t>정수</t>
         </is>
       </c>
       <c r="I55" s="5" t="inlineStr">
@@ -3502,37 +3506,37 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>heightMinCm</t>
+          <t>romSetting</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>키최소</t>
+          <t>가동 범위</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Height Min</t>
+          <t>Range of Motion</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t>추천매칭</t>
-        </is>
-      </c>
-      <c r="F56" s="8" t="inlineStr">
-        <is>
-          <t>내부용</t>
-        </is>
-      </c>
-      <c r="G56" s="7" t="inlineStr">
-        <is>
-          <t>필수</t>
+          <t>추천결과/기록/비교</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>표시중</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>조건부</t>
         </is>
       </c>
       <c r="H56" s="5" t="inlineStr">
         <is>
-          <t>숫자(cm)</t>
+          <t>문자열</t>
         </is>
       </c>
       <c r="I56" s="5" t="inlineStr">
@@ -3540,7 +3544,11 @@
           <t>05_추천설정_팁주의</t>
         </is>
       </c>
-      <c r="J56" s="5" t="inlineStr"/>
+      <c r="J56" s="5" t="inlineStr">
+        <is>
+          <t>최대/부분/반/짧게/가변</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
@@ -3550,37 +3558,37 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>heightMaxCm</t>
+          <t>recommendedWeightKg</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>키최대</t>
+          <t>추천 중량</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>Height Max</t>
+          <t>Recommended Weight</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t>추천매칭</t>
-        </is>
-      </c>
-      <c r="F57" s="8" t="inlineStr">
-        <is>
-          <t>내부용</t>
-        </is>
-      </c>
-      <c r="G57" s="7" t="inlineStr">
-        <is>
-          <t>필수</t>
+          <t>추천결과/기록/비교</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>표시중</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>권장</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr">
         <is>
-          <t>숫자(cm)</t>
+          <t>숫자(kg)</t>
         </is>
       </c>
       <c r="I57" s="5" t="inlineStr">
@@ -3593,27 +3601,27 @@
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>추천팁</t>
+          <t>추천설정</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>tips.ko</t>
+          <t>recommendedRepsMin</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>운동팁(한글)</t>
+          <t>추천횟수최소</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Workout Tips KO</t>
+          <t>Reps Min</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t>추천결과/휴식음성</t>
+          <t>추천결과</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">
@@ -3623,12 +3631,12 @@
       </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
-          <t>권장</t>
+          <t>선택</t>
         </is>
       </c>
       <c r="H58" s="5" t="inlineStr">
         <is>
-          <t>줄바꿈 문장목록</t>
+          <t>정수</t>
         </is>
       </c>
       <c r="I58" s="5" t="inlineStr">
@@ -3638,29 +3646,29 @@
       </c>
       <c r="J58" s="5" t="inlineStr">
         <is>
-          <t>TTS 핵심</t>
+          <t>없으면 목표기반 계산</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>추천팁</t>
+          <t>추천설정</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>tips.en</t>
+          <t>recommendedRepsMax</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>운동팁(영문)</t>
+          <t>추천횟수최대</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>Workout Tips EN</t>
+          <t>Reps Max</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -3675,12 +3683,12 @@
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>권장</t>
+          <t>선택</t>
         </is>
       </c>
       <c r="H59" s="5" t="inlineStr">
         <is>
-          <t>줄바꿈 문장목록</t>
+          <t>정수</t>
         </is>
       </c>
       <c r="I59" s="5" t="inlineStr">
@@ -3693,42 +3701,42 @@
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>추천팁</t>
+          <t>추천설정</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>warnings.ko</t>
+          <t>gender</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>주의(한글)</t>
+          <t>성별조건</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>Warnings KO</t>
+          <t>Gender</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t>추천결과/휴식음성</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="inlineStr">
-        <is>
-          <t>표시중</t>
-        </is>
-      </c>
-      <c r="G60" s="5" t="inlineStr">
-        <is>
-          <t>권장</t>
+          <t>추천매칭</t>
+        </is>
+      </c>
+      <c r="F60" s="8" t="inlineStr">
+        <is>
+          <t>내부용</t>
+        </is>
+      </c>
+      <c r="G60" s="7" t="inlineStr">
+        <is>
+          <t>필수</t>
         </is>
       </c>
       <c r="H60" s="5" t="inlineStr">
         <is>
-          <t>줄바꿈 문장목록</t>
+          <t>male/female</t>
         </is>
       </c>
       <c r="I60" s="5" t="inlineStr">
@@ -3736,51 +3744,47 @@
           <t>05_추천설정_팁주의</t>
         </is>
       </c>
-      <c r="J60" s="5" t="inlineStr">
-        <is>
-          <t>TTS 핵심</t>
-        </is>
-      </c>
+      <c r="J60" s="5" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>추천팁</t>
+          <t>추천설정</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>warnings.en</t>
+          <t>experienceLevel</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>주의(영문)</t>
+          <t>경험레벨조건</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Warnings EN</t>
+          <t>Experience</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>추천결과</t>
-        </is>
-      </c>
-      <c r="F61" s="6" t="inlineStr">
-        <is>
-          <t>표시중</t>
-        </is>
-      </c>
-      <c r="G61" s="5" t="inlineStr">
-        <is>
-          <t>권장</t>
+          <t>추천매칭</t>
+        </is>
+      </c>
+      <c r="F61" s="8" t="inlineStr">
+        <is>
+          <t>내부용</t>
+        </is>
+      </c>
+      <c r="G61" s="7" t="inlineStr">
+        <is>
+          <t>필수</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr">
         <is>
-          <t>줄바꿈 문장목록</t>
+          <t>beginner/intermediate/advanced</t>
         </is>
       </c>
       <c r="I61" s="5" t="inlineStr">
@@ -3793,131 +3797,123 @@
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>영상</t>
+          <t>추천설정</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>youtubeId</t>
+          <t>heightMinCm</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>유튜브ID</t>
+          <t>키최소</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>YouTube ID</t>
+          <t>Height Min</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>추천결과(예정)</t>
-        </is>
-      </c>
-      <c r="F62" s="9" t="inlineStr">
-        <is>
-          <t>데이터만</t>
-        </is>
-      </c>
-      <c r="G62" s="5" t="inlineStr">
-        <is>
-          <t>선택</t>
+          <t>추천매칭</t>
+        </is>
+      </c>
+      <c r="F62" s="8" t="inlineStr">
+        <is>
+          <t>내부용</t>
+        </is>
+      </c>
+      <c r="G62" s="7" t="inlineStr">
+        <is>
+          <t>필수</t>
         </is>
       </c>
       <c r="H62" s="5" t="inlineStr">
         <is>
-          <t>문자열</t>
+          <t>숫자(cm)</t>
         </is>
       </c>
       <c r="I62" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J62" s="5" t="inlineStr">
-        <is>
-          <t>현재 UI 없음</t>
-        </is>
-      </c>
+          <t>05_추천설정_팁주의</t>
+        </is>
+      </c>
+      <c r="J62" s="5" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>영상</t>
+          <t>추천설정</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>videoUrl</t>
+          <t>heightMaxCm</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>머신영상URL</t>
+          <t>키최대</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>Video URL</t>
+          <t>Height Max</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t>상세(예정)</t>
-        </is>
-      </c>
-      <c r="F63" s="9" t="inlineStr">
-        <is>
-          <t>데이터만</t>
-        </is>
-      </c>
-      <c r="G63" s="5" t="inlineStr">
-        <is>
-          <t>선택</t>
+          <t>추천매칭</t>
+        </is>
+      </c>
+      <c r="F63" s="8" t="inlineStr">
+        <is>
+          <t>내부용</t>
+        </is>
+      </c>
+      <c r="G63" s="7" t="inlineStr">
+        <is>
+          <t>필수</t>
         </is>
       </c>
       <c r="H63" s="5" t="inlineStr">
         <is>
-          <t>URL</t>
+          <t>숫자(cm)</t>
         </is>
       </c>
       <c r="I63" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J63" s="5" t="inlineStr">
-        <is>
-          <t>현재 UI 없음</t>
-        </is>
-      </c>
+          <t>05_추천설정_팁주의</t>
+        </is>
+      </c>
+      <c r="J63" s="5" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>헬스장머신</t>
+          <t>추천팁</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>machineCode</t>
+          <t>tips.ko</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>머신코드</t>
+          <t>운동팁(한글)</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>Machine Code</t>
+          <t>Workout Tips KO</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>헬스장상세</t>
+          <t>추천결과/휴식음성</t>
         </is>
       </c>
       <c r="F64" s="6" t="inlineStr">
@@ -3925,47 +3921,51 @@
           <t>표시중</t>
         </is>
       </c>
-      <c r="G64" s="7" t="inlineStr">
-        <is>
-          <t>필수</t>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>권장</t>
         </is>
       </c>
       <c r="H64" s="5" t="inlineStr">
         <is>
-          <t>문자열</t>
+          <t>줄바꿈 문장목록</t>
         </is>
       </c>
       <c r="I64" s="5" t="inlineStr">
         <is>
-          <t>06_헬스장보유머신</t>
-        </is>
-      </c>
-      <c r="J64" s="5" t="inlineStr"/>
+          <t>05_추천설정_팁주의</t>
+        </is>
+      </c>
+      <c r="J64" s="5" t="inlineStr">
+        <is>
+          <t>TTS 핵심</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>헬스장머신</t>
+          <t>추천팁</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>machineName</t>
+          <t>tips.en</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>머신표시명</t>
+          <t>운동팁(영문)</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>Machine Name</t>
+          <t>Workout Tips EN</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>헬스장상세/재고</t>
+          <t>추천결과</t>
         </is>
       </c>
       <c r="F65" s="6" t="inlineStr">
@@ -3973,19 +3973,19 @@
           <t>표시중</t>
         </is>
       </c>
-      <c r="G65" s="7" t="inlineStr">
-        <is>
-          <t>필수</t>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>권장</t>
         </is>
       </c>
       <c r="H65" s="5" t="inlineStr">
         <is>
-          <t>문자열</t>
+          <t>줄바꿈 문장목록</t>
         </is>
       </c>
       <c r="I65" s="5" t="inlineStr">
         <is>
-          <t>06_헬스장보유머신</t>
+          <t>05_추천설정_팁주의</t>
         </is>
       </c>
       <c r="J65" s="5" t="inlineStr"/>
@@ -3993,27 +3993,27 @@
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>헬스장머신</t>
+          <t>추천팁</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>quantity</t>
+          <t>warnings.ko</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>대수</t>
+          <t>주의(한글)</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>Quantity</t>
+          <t>Warnings KO</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t>헬스장상세</t>
+          <t>추천결과/휴식음성</t>
         </is>
       </c>
       <c r="F66" s="6" t="inlineStr">
@@ -4023,49 +4023,49 @@
       </c>
       <c r="G66" s="5" t="inlineStr">
         <is>
-          <t>선택</t>
+          <t>권장</t>
         </is>
       </c>
       <c r="H66" s="5" t="inlineStr">
         <is>
-          <t>정수</t>
+          <t>줄바꿈 문장목록</t>
         </is>
       </c>
       <c r="I66" s="5" t="inlineStr">
         <is>
-          <t>06_헬스장보유머신</t>
+          <t>05_추천설정_팁주의</t>
         </is>
       </c>
       <c r="J66" s="5" t="inlineStr">
         <is>
-          <t>대</t>
+          <t>TTS 핵심</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>헬스장머신</t>
+          <t>추천팁</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>floorZone</t>
+          <t>warnings.en</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>위치구역</t>
+          <t>주의(영문)</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>Floor Zone</t>
+          <t>Warnings EN</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>헬스장상세</t>
+          <t>추천결과</t>
         </is>
       </c>
       <c r="F67" s="6" t="inlineStr">
@@ -4075,102 +4075,102 @@
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>선택</t>
+          <t>권장</t>
         </is>
       </c>
       <c r="H67" s="5" t="inlineStr">
         <is>
-          <t>문자열</t>
+          <t>줄바꿈 문장목록</t>
         </is>
       </c>
       <c r="I67" s="5" t="inlineStr">
         <is>
-          <t>06_헬스장보유머신</t>
-        </is>
-      </c>
-      <c r="J67" s="5" t="inlineStr">
-        <is>
-          <t>예: 1층 하체존</t>
-        </is>
-      </c>
+          <t>05_추천설정_팁주의</t>
+        </is>
+      </c>
+      <c r="J67" s="5" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>헬스장머신</t>
+          <t>영상</t>
         </is>
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>isAvailable</t>
+          <t>youtubeId</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>사용가능</t>
+          <t>유튜브ID</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>Available</t>
+          <t>YouTube ID</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t>헬스장상세</t>
-        </is>
-      </c>
-      <c r="F68" s="6" t="inlineStr">
-        <is>
-          <t>표시중</t>
-        </is>
-      </c>
-      <c r="G68" s="7" t="inlineStr">
-        <is>
-          <t>필수</t>
+          <t>추천결과(예정)</t>
+        </is>
+      </c>
+      <c r="F68" s="9" t="inlineStr">
+        <is>
+          <t>데이터만</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>선택</t>
         </is>
       </c>
       <c r="H68" s="5" t="inlineStr">
         <is>
-          <t>TRUE/FALSE</t>
+          <t>문자열</t>
         </is>
       </c>
       <c r="I68" s="5" t="inlineStr">
         <is>
-          <t>06_헬스장보유머신</t>
-        </is>
-      </c>
-      <c r="J68" s="5" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J68" s="5" t="inlineStr">
+        <is>
+          <t>현재 UI 없음</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>헬스장머신</t>
+          <t>영상</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>notes</t>
+          <t>videoUrl</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>메모</t>
+          <t>머신영상URL</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Video URL</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t>헬스장상세(비가용시)</t>
-        </is>
-      </c>
-      <c r="F69" s="6" t="inlineStr">
-        <is>
-          <t>표시중</t>
+          <t>상세(예정)</t>
+        </is>
+      </c>
+      <c r="F69" s="9" t="inlineStr">
+        <is>
+          <t>데이터만</t>
         </is>
       </c>
       <c r="G69" s="5" t="inlineStr">
@@ -4180,40 +4180,44 @@
       </c>
       <c r="H69" s="5" t="inlineStr">
         <is>
-          <t>문자열</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="I69" s="5" t="inlineStr">
         <is>
-          <t>06_헬스장보유머신</t>
-        </is>
-      </c>
-      <c r="J69" s="5" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J69" s="5" t="inlineStr">
+        <is>
+          <t>현재 UI 없음</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>사용자</t>
+          <t>헬스장머신</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>personalTipMemo</t>
+          <t>machineCode</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>나만의 팁 메모장</t>
+          <t>머신코드</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>My tip notebook</t>
+          <t>Machine Code</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t>운동기록</t>
+          <t>헬스장상세</t>
         </is>
       </c>
       <c r="F70" s="6" t="inlineStr">
@@ -4221,74 +4225,370 @@
           <t>표시중</t>
         </is>
       </c>
-      <c r="G70" s="5" t="inlineStr">
-        <is>
-          <t>선택</t>
+      <c r="G70" s="7" t="inlineStr">
+        <is>
+          <t>필수</t>
         </is>
       </c>
       <c r="H70" s="5" t="inlineStr">
         <is>
-          <t>사용자입력</t>
+          <t>문자열</t>
         </is>
       </c>
       <c r="I70" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J70" s="5" t="inlineStr">
-        <is>
-          <t>카탈로그 작성대상 아님</t>
-        </is>
-      </c>
+          <t>06_헬스장보유머신</t>
+        </is>
+      </c>
+      <c r="J70" s="5" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
+          <t>헬스장머신</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>machineName</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>머신표시명</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>Machine Name</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>헬스장상세/재고</t>
+        </is>
+      </c>
+      <c r="F71" s="6" t="inlineStr">
+        <is>
+          <t>표시중</t>
+        </is>
+      </c>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>필수</t>
+        </is>
+      </c>
+      <c r="H71" s="5" t="inlineStr">
+        <is>
+          <t>문자열</t>
+        </is>
+      </c>
+      <c r="I71" s="5" t="inlineStr">
+        <is>
+          <t>06_헬스장보유머신</t>
+        </is>
+      </c>
+      <c r="J71" s="5" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>헬스장머신</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>대수</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>헬스장상세</t>
+        </is>
+      </c>
+      <c r="F72" s="6" t="inlineStr">
+        <is>
+          <t>표시중</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>선택</t>
+        </is>
+      </c>
+      <c r="H72" s="5" t="inlineStr">
+        <is>
+          <t>정수</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>06_헬스장보유머신</t>
+        </is>
+      </c>
+      <c r="J72" s="5" t="inlineStr">
+        <is>
+          <t>대</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>헬스장머신</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>floorZone</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>위치구역</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>Floor Zone</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>헬스장상세</t>
+        </is>
+      </c>
+      <c r="F73" s="6" t="inlineStr">
+        <is>
+          <t>표시중</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>선택</t>
+        </is>
+      </c>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
+          <t>문자열</t>
+        </is>
+      </c>
+      <c r="I73" s="5" t="inlineStr">
+        <is>
+          <t>06_헬스장보유머신</t>
+        </is>
+      </c>
+      <c r="J73" s="5" t="inlineStr">
+        <is>
+          <t>예: 1층 하체존</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>헬스장머신</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>isAvailable</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>사용가능</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>헬스장상세</t>
+        </is>
+      </c>
+      <c r="F74" s="6" t="inlineStr">
+        <is>
+          <t>표시중</t>
+        </is>
+      </c>
+      <c r="G74" s="7" t="inlineStr">
+        <is>
+          <t>필수</t>
+        </is>
+      </c>
+      <c r="H74" s="5" t="inlineStr">
+        <is>
+          <t>TRUE/FALSE</t>
+        </is>
+      </c>
+      <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>06_헬스장보유머신</t>
+        </is>
+      </c>
+      <c r="J74" s="5" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>헬스장머신</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>메모</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>헬스장상세(비가용시)</t>
+        </is>
+      </c>
+      <c r="F75" s="6" t="inlineStr">
+        <is>
+          <t>표시중</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>선택</t>
+        </is>
+      </c>
+      <c r="H75" s="5" t="inlineStr">
+        <is>
+          <t>문자열</t>
+        </is>
+      </c>
+      <c r="I75" s="5" t="inlineStr">
+        <is>
+          <t>06_헬스장보유머신</t>
+        </is>
+      </c>
+      <c r="J75" s="5" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>사용자</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>personalTipMemo</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>나만의 팁 메모장</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>My tip notebook</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>운동기록</t>
+        </is>
+      </c>
+      <c r="F76" s="6" t="inlineStr">
+        <is>
+          <t>표시중</t>
+        </is>
+      </c>
+      <c r="G76" s="5" t="inlineStr">
+        <is>
+          <t>선택</t>
+        </is>
+      </c>
+      <c r="H76" s="5" t="inlineStr">
+        <is>
+          <t>사용자입력</t>
+        </is>
+      </c>
+      <c r="I76" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J76" s="5" t="inlineStr">
+        <is>
+          <t>카탈로그 작성대상 아님</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
           <t>요청게시판</t>
         </is>
       </c>
-      <c r="B71" s="5" t="inlineStr">
+      <c r="B77" s="5" t="inlineStr">
         <is>
           <t>brandName/machineName/description</t>
         </is>
       </c>
-      <c r="C71" s="5" t="inlineStr">
+      <c r="C77" s="5" t="inlineStr">
         <is>
           <t>브랜드/기구명/설명</t>
         </is>
       </c>
-      <c r="D71" s="5" t="inlineStr">
+      <c r="D77" s="5" t="inlineStr">
         <is>
           <t>Request fields</t>
         </is>
       </c>
-      <c r="E71" s="5" t="inlineStr">
+      <c r="E77" s="5" t="inlineStr">
         <is>
           <t>머신요청게시판</t>
         </is>
       </c>
-      <c r="F71" s="6" t="inlineStr">
+      <c r="F77" s="6" t="inlineStr">
         <is>
           <t>표시중</t>
         </is>
       </c>
-      <c r="G71" s="5" t="inlineStr">
+      <c r="G77" s="5" t="inlineStr">
         <is>
           <t>부분필수</t>
         </is>
       </c>
-      <c r="H71" s="5" t="inlineStr">
+      <c r="H77" s="5" t="inlineStr">
         <is>
           <t>자유텍스트</t>
         </is>
       </c>
-      <c r="I71" s="5" t="inlineStr">
+      <c r="I77" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J71" s="5" t="inlineStr">
+      <c r="J77" s="5" t="inlineStr">
         <is>
           <t>카탈로그 아님</t>
         </is>
@@ -4621,7 +4921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z17"/>
+  <dimension ref="A1:AF17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4745,40 +5045,70 @@
       </c>
       <c r="S1" s="4" t="inlineStr">
         <is>
+          <t>intermediateTips_ko (줄바꿈)</t>
+        </is>
+      </c>
+      <c r="T1" s="4" t="inlineStr">
+        <is>
+          <t>intermediateTips_en (줄바꿈)</t>
+        </is>
+      </c>
+      <c r="U1" s="4" t="inlineStr">
+        <is>
+          <t>advancedTips_ko (줄바꿈)</t>
+        </is>
+      </c>
+      <c r="V1" s="4" t="inlineStr">
+        <is>
+          <t>advancedTips_en (줄바꿈)</t>
+        </is>
+      </c>
+      <c r="W1" s="4" t="inlineStr">
+        <is>
+          <t>proTips_ko (줄바꿈)</t>
+        </is>
+      </c>
+      <c r="X1" s="4" t="inlineStr">
+        <is>
+          <t>proTips_en (줄바꿈)</t>
+        </is>
+      </c>
+      <c r="Y1" s="4" t="inlineStr">
+        <is>
           <t>recommendedExperience</t>
         </is>
       </c>
-      <c r="T1" s="4" t="inlineStr">
+      <c r="Z1" s="4" t="inlineStr">
         <is>
           <t>hasSeat*</t>
         </is>
       </c>
-      <c r="U1" s="4" t="inlineStr">
+      <c r="AA1" s="4" t="inlineStr">
         <is>
           <t>hasBackPad*</t>
         </is>
       </c>
-      <c r="V1" s="4" t="inlineStr">
+      <c r="AB1" s="4" t="inlineStr">
         <is>
           <t>hasFootPlate*</t>
         </is>
       </c>
-      <c r="W1" s="4" t="inlineStr">
+      <c r="AC1" s="4" t="inlineStr">
         <is>
           <t>hasHandle*</t>
         </is>
       </c>
-      <c r="X1" s="4" t="inlineStr">
+      <c r="AD1" s="4" t="inlineStr">
         <is>
           <t>romType</t>
         </is>
       </c>
-      <c r="Y1" s="4" t="inlineStr">
+      <c r="AE1" s="4" t="inlineStr">
         <is>
           <t>isActive*</t>
         </is>
       </c>
-      <c r="Z1" s="4" t="inlineStr">
+      <c r="AF1" s="4" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
@@ -5015,6 +5345,12 @@
       <c r="X3" s="5" t="inlineStr"/>
       <c r="Y3" s="5" t="inlineStr"/>
       <c r="Z3" s="5" t="inlineStr"/>
+      <c r="AA3" s="5" t="inlineStr"/>
+      <c r="AB3" s="5" t="inlineStr"/>
+      <c r="AC3" s="5" t="inlineStr"/>
+      <c r="AD3" s="5" t="inlineStr"/>
+      <c r="AE3" s="5" t="inlineStr"/>
+      <c r="AF3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr"/>
@@ -5043,6 +5379,12 @@
       <c r="X4" s="5" t="inlineStr"/>
       <c r="Y4" s="5" t="inlineStr"/>
       <c r="Z4" s="5" t="inlineStr"/>
+      <c r="AA4" s="5" t="inlineStr"/>
+      <c r="AB4" s="5" t="inlineStr"/>
+      <c r="AC4" s="5" t="inlineStr"/>
+      <c r="AD4" s="5" t="inlineStr"/>
+      <c r="AE4" s="5" t="inlineStr"/>
+      <c r="AF4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr"/>
@@ -5071,6 +5413,12 @@
       <c r="X5" s="5" t="inlineStr"/>
       <c r="Y5" s="5" t="inlineStr"/>
       <c r="Z5" s="5" t="inlineStr"/>
+      <c r="AA5" s="5" t="inlineStr"/>
+      <c r="AB5" s="5" t="inlineStr"/>
+      <c r="AC5" s="5" t="inlineStr"/>
+      <c r="AD5" s="5" t="inlineStr"/>
+      <c r="AE5" s="5" t="inlineStr"/>
+      <c r="AF5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr"/>
@@ -5099,6 +5447,12 @@
       <c r="X6" s="5" t="inlineStr"/>
       <c r="Y6" s="5" t="inlineStr"/>
       <c r="Z6" s="5" t="inlineStr"/>
+      <c r="AA6" s="5" t="inlineStr"/>
+      <c r="AB6" s="5" t="inlineStr"/>
+      <c r="AC6" s="5" t="inlineStr"/>
+      <c r="AD6" s="5" t="inlineStr"/>
+      <c r="AE6" s="5" t="inlineStr"/>
+      <c r="AF6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr"/>
@@ -5127,6 +5481,12 @@
       <c r="X7" s="5" t="inlineStr"/>
       <c r="Y7" s="5" t="inlineStr"/>
       <c r="Z7" s="5" t="inlineStr"/>
+      <c r="AA7" s="5" t="inlineStr"/>
+      <c r="AB7" s="5" t="inlineStr"/>
+      <c r="AC7" s="5" t="inlineStr"/>
+      <c r="AD7" s="5" t="inlineStr"/>
+      <c r="AE7" s="5" t="inlineStr"/>
+      <c r="AF7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr"/>
@@ -5155,6 +5515,12 @@
       <c r="X8" s="5" t="inlineStr"/>
       <c r="Y8" s="5" t="inlineStr"/>
       <c r="Z8" s="5" t="inlineStr"/>
+      <c r="AA8" s="5" t="inlineStr"/>
+      <c r="AB8" s="5" t="inlineStr"/>
+      <c r="AC8" s="5" t="inlineStr"/>
+      <c r="AD8" s="5" t="inlineStr"/>
+      <c r="AE8" s="5" t="inlineStr"/>
+      <c r="AF8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr"/>
@@ -5183,6 +5549,12 @@
       <c r="X9" s="5" t="inlineStr"/>
       <c r="Y9" s="5" t="inlineStr"/>
       <c r="Z9" s="5" t="inlineStr"/>
+      <c r="AA9" s="5" t="inlineStr"/>
+      <c r="AB9" s="5" t="inlineStr"/>
+      <c r="AC9" s="5" t="inlineStr"/>
+      <c r="AD9" s="5" t="inlineStr"/>
+      <c r="AE9" s="5" t="inlineStr"/>
+      <c r="AF9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr"/>
@@ -5211,6 +5583,12 @@
       <c r="X10" s="5" t="inlineStr"/>
       <c r="Y10" s="5" t="inlineStr"/>
       <c r="Z10" s="5" t="inlineStr"/>
+      <c r="AA10" s="5" t="inlineStr"/>
+      <c r="AB10" s="5" t="inlineStr"/>
+      <c r="AC10" s="5" t="inlineStr"/>
+      <c r="AD10" s="5" t="inlineStr"/>
+      <c r="AE10" s="5" t="inlineStr"/>
+      <c r="AF10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr"/>
@@ -5239,6 +5617,12 @@
       <c r="X11" s="5" t="inlineStr"/>
       <c r="Y11" s="5" t="inlineStr"/>
       <c r="Z11" s="5" t="inlineStr"/>
+      <c r="AA11" s="5" t="inlineStr"/>
+      <c r="AB11" s="5" t="inlineStr"/>
+      <c r="AC11" s="5" t="inlineStr"/>
+      <c r="AD11" s="5" t="inlineStr"/>
+      <c r="AE11" s="5" t="inlineStr"/>
+      <c r="AF11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr"/>
@@ -5267,6 +5651,12 @@
       <c r="X12" s="5" t="inlineStr"/>
       <c r="Y12" s="5" t="inlineStr"/>
       <c r="Z12" s="5" t="inlineStr"/>
+      <c r="AA12" s="5" t="inlineStr"/>
+      <c r="AB12" s="5" t="inlineStr"/>
+      <c r="AC12" s="5" t="inlineStr"/>
+      <c r="AD12" s="5" t="inlineStr"/>
+      <c r="AE12" s="5" t="inlineStr"/>
+      <c r="AF12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr"/>
@@ -5295,6 +5685,12 @@
       <c r="X13" s="5" t="inlineStr"/>
       <c r="Y13" s="5" t="inlineStr"/>
       <c r="Z13" s="5" t="inlineStr"/>
+      <c r="AA13" s="5" t="inlineStr"/>
+      <c r="AB13" s="5" t="inlineStr"/>
+      <c r="AC13" s="5" t="inlineStr"/>
+      <c r="AD13" s="5" t="inlineStr"/>
+      <c r="AE13" s="5" t="inlineStr"/>
+      <c r="AF13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr"/>
@@ -5323,6 +5719,12 @@
       <c r="X14" s="5" t="inlineStr"/>
       <c r="Y14" s="5" t="inlineStr"/>
       <c r="Z14" s="5" t="inlineStr"/>
+      <c r="AA14" s="5" t="inlineStr"/>
+      <c r="AB14" s="5" t="inlineStr"/>
+      <c r="AC14" s="5" t="inlineStr"/>
+      <c r="AD14" s="5" t="inlineStr"/>
+      <c r="AE14" s="5" t="inlineStr"/>
+      <c r="AF14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr"/>
@@ -5351,6 +5753,12 @@
       <c r="X15" s="5" t="inlineStr"/>
       <c r="Y15" s="5" t="inlineStr"/>
       <c r="Z15" s="5" t="inlineStr"/>
+      <c r="AA15" s="5" t="inlineStr"/>
+      <c r="AB15" s="5" t="inlineStr"/>
+      <c r="AC15" s="5" t="inlineStr"/>
+      <c r="AD15" s="5" t="inlineStr"/>
+      <c r="AE15" s="5" t="inlineStr"/>
+      <c r="AF15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr"/>
@@ -5379,6 +5787,12 @@
       <c r="X16" s="5" t="inlineStr"/>
       <c r="Y16" s="5" t="inlineStr"/>
       <c r="Z16" s="5" t="inlineStr"/>
+      <c r="AA16" s="5" t="inlineStr"/>
+      <c r="AB16" s="5" t="inlineStr"/>
+      <c r="AC16" s="5" t="inlineStr"/>
+      <c r="AD16" s="5" t="inlineStr"/>
+      <c r="AE16" s="5" t="inlineStr"/>
+      <c r="AF16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr"/>
@@ -5407,9 +5821,15 @@
       <c r="X17" s="5" t="inlineStr"/>
       <c r="Y17" s="5" t="inlineStr"/>
       <c r="Z17" s="5" t="inlineStr"/>
+      <c r="AA17" s="5" t="inlineStr"/>
+      <c r="AB17" s="5" t="inlineStr"/>
+      <c r="AC17" s="5" t="inlineStr"/>
+      <c r="AD17" s="5" t="inlineStr"/>
+      <c r="AE17" s="5" t="inlineStr"/>
+      <c r="AF17" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z1"/>
+  <autoFilter ref="A1:AF1"/>
   <dataValidations count="8">
     <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"chest,back,legs,shoulders,biceps,triceps,core,full_body"</formula1>

</xml_diff>